<commit_message>
Add DTW IT Center PM Dashboard; fix construction budget category totals
- New Streamlit dashboard (dtw-pm-dashboard/) operationalizing the PM
  Toolkit's schedule, budget, risk, stakeholder, and closeout data into
  an interactive portfolio rollup, Gantt view, budget variance charts,
  risk heatmap, stakeholder power/interest grid, and a lessons-learned
  page.
- Fixed construction project budget categories in the PM Tracking
  Workbook and Status/Closeout Report: they previously summed to
  $5.42M against a stated $4.25M GMP total; rebalanced so all
  categories (including contingency) reconcile to $4,250,000 exactly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dtw-it-center-pm-toolkit/01-construction-infrastructure-project/02_PM_Tracking_Workbook.xlsx
+++ b/dtw-it-center-pm-toolkit/01-construction-infrastructure-project/02_PM_Tracking_Workbook.xlsx
@@ -1809,13 +1809,13 @@
         <v>33</v>
       </c>
       <c r="B3" s="12" t="n">
-        <v>780000</v>
+        <v>650000</v>
       </c>
       <c r="C3" s="12" t="n">
-        <v>780000</v>
+        <v>650000</v>
       </c>
       <c r="D3" s="12" t="n">
-        <v>775000</v>
+        <v>645000</v>
       </c>
       <c r="E3" s="12" t="n">
         <f aca="false">D3-B3</f>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="F3" s="13" t="n">
         <f aca="false">IFERROR(D3/B3,0)</f>
-        <v>0.993589743589744</v>
+        <v>0.992307692307692</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>27</v>
@@ -1834,21 +1834,21 @@
         <v>88</v>
       </c>
       <c r="B4" s="14" t="n">
-        <v>1020000</v>
+        <v>850000</v>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1020000</v>
+        <v>850000</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1005000</v>
+        <v>838000</v>
       </c>
       <c r="E4" s="14" t="n">
         <f aca="false">D4-B4</f>
-        <v>-15000</v>
+        <v>-12000</v>
       </c>
       <c r="F4" s="15" t="n">
         <f aca="false">IFERROR(D4/B4,0)</f>
-        <v>0.985294117647059</v>
+        <v>0.985882352941176</v>
       </c>
       <c r="G4" s="11" t="s">
         <v>27</v>
@@ -1859,21 +1859,21 @@
         <v>89</v>
       </c>
       <c r="B5" s="12" t="n">
-        <v>1450000</v>
+        <v>1000000</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>1310000</v>
+        <v>903000</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>1180000</v>
+        <v>810000</v>
       </c>
       <c r="E5" s="12" t="n">
         <f aca="false">D5-B5</f>
-        <v>-270000</v>
+        <v>-190000</v>
       </c>
       <c r="F5" s="13" t="n">
         <f aca="false">IFERROR(D5/B5,0)</f>
-        <v>0.813793103448276</v>
+        <v>0.81</v>
       </c>
       <c r="G5" s="10" t="s">
         <v>90</v>
@@ -1884,21 +1884,21 @@
         <v>91</v>
       </c>
       <c r="B6" s="14" t="n">
-        <v>980000</v>
+        <v>780000</v>
       </c>
       <c r="C6" s="14" t="n">
-        <v>720000</v>
+        <v>573000</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>640000</v>
+        <v>507000</v>
       </c>
       <c r="E6" s="14" t="n">
         <f aca="false">D6-B6</f>
-        <v>-340000</v>
+        <v>-273000</v>
       </c>
       <c r="F6" s="15" t="n">
         <f aca="false">IFERROR(D6/B6,0)</f>
-        <v>0.653061224489796</v>
+        <v>0.65</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>92</v>
@@ -1909,21 +1909,21 @@
         <v>93</v>
       </c>
       <c r="B7" s="12" t="n">
-        <v>210000</v>
+        <v>170000</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>205000</v>
+        <v>166000</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>198000</v>
+        <v>160000</v>
       </c>
       <c r="E7" s="12" t="n">
         <f aca="false">D7-B7</f>
-        <v>-12000</v>
+        <v>-10000</v>
       </c>
       <c r="F7" s="13" t="n">
         <f aca="false">IFERROR(D7/B7,0)</f>
-        <v>0.942857142857143</v>
+        <v>0.941176470588235</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>27</v>
@@ -1934,7 +1934,7 @@
         <v>94</v>
       </c>
       <c r="B8" s="14" t="n">
-        <v>260000</v>
+        <v>210000</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>0</v>
@@ -1944,7 +1944,7 @@
       </c>
       <c r="E8" s="14" t="n">
         <f aca="false">D8-B8</f>
-        <v>-260000</v>
+        <v>-210000</v>
       </c>
       <c r="F8" s="15" t="n">
         <f aca="false">IFERROR(D8/B8,0)</f>
@@ -1959,7 +1959,7 @@
         <v>96</v>
       </c>
       <c r="B9" s="12" t="n">
-        <v>190000</v>
+        <v>150000</v>
       </c>
       <c r="C9" s="12" t="n">
         <v>0</v>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="E9" s="12" t="n">
         <f aca="false">D9-B9</f>
-        <v>-190000</v>
+        <v>-150000</v>
       </c>
       <c r="F9" s="13" t="n">
         <f aca="false">IFERROR(D9/B9,0)</f>
@@ -1984,13 +1984,13 @@
         <v>97</v>
       </c>
       <c r="B10" s="14" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="C10" s="14" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>58000</v>
+        <v>48000</v>
       </c>
       <c r="E10" s="14" t="n">
         <f aca="false">D10-B10</f>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="F10" s="15" t="n">
         <f aca="false">IFERROR(D10/B10,0)</f>
-        <v>0.966666666666667</v>
+        <v>0.96</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>27</v>
@@ -2009,7 +2009,7 @@
         <v>68</v>
       </c>
       <c r="B11" s="12" t="n">
-        <v>130000</v>
+        <v>50000</v>
       </c>
       <c r="C11" s="12" t="n">
         <v>0</v>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">D11-B11</f>
-        <v>-130000</v>
+        <v>-50000</v>
       </c>
       <c r="F11" s="13" t="n">
         <f aca="false">IFERROR(D11/B11,0)</f>
@@ -2060,23 +2060,23 @@
       </c>
       <c r="B13" s="17" t="n">
         <f aca="false">SUM(B3:B12)</f>
-        <v>5420000</v>
+        <v>4250000</v>
       </c>
       <c r="C13" s="17" t="n">
         <f aca="false">SUM(C3:C12)</f>
-        <v>4156000</v>
+        <v>3253000</v>
       </c>
       <c r="D13" s="17" t="n">
         <f aca="false">SUM(D3:D12)</f>
-        <v>3917000</v>
+        <v>3069000</v>
       </c>
       <c r="E13" s="17" t="n">
         <f aca="false">D13-B13</f>
-        <v>-1503000</v>
+        <v>-1181000</v>
       </c>
       <c r="F13" s="18" t="n">
         <f aca="false">IFERROR(D13/B13,0)</f>
-        <v>0.722693726937269</v>
+        <v>0.722117647058824</v>
       </c>
       <c r="G13" s="16"/>
     </row>

</xml_diff>

<commit_message>
Add Quality Management to PM toolkit and dashboard
Fills the PMBOK quality-management gap identified on review: each
project's Charter now includes a Quality Management Plan (standards,
QA activities, QC/inspection & test checkpoints), each PM Tracking
Workbook has a Quality_Checklist tab, and the dashboard has a new
Quality Management page mirroring both. Applied to the blank
templates and both worked example projects.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dtw-it-center-pm-toolkit/01-construction-infrastructure-project/02_PM_Tracking_Workbook.xlsx
+++ b/dtw-it-center-pm-toolkit/01-construction-infrastructure-project/02_PM_Tracking_Workbook.xlsx
@@ -11,11 +11,12 @@
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="WBS_Schedule" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Budget_Tracker" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="RACI_Matrix" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Stakeholder_Register" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Risk_Register" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Issue_Change_Log" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Vendor_Contractor_Register" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Quality_Checklist" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="RACI_Matrix" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Stakeholder_Register" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Risk_Register" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Issue_Change_Log" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Vendor_Contractor_Register" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="260">
   <si>
     <t xml:space="preserve">IT Center Data Center &amp; NOC Build-Out — PM Tracking Workbook</t>
   </si>
@@ -332,6 +333,81 @@
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
+    <t xml:space="preserve">Quality Control Checklist  (deliverable/checkpoint acceptance tracking)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checkpoint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acceptance Criteria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inspection Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foundation / sitework inspection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Structural</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Passes AHJ foundation inspection; geotechnical sign-off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AHJ inspection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEP rough-in inspection (electrical, mechanical, fire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Passes AHJ rough-in inspection; matches approved design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GC / Subcontractors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level 1-2 Commissioning (equipment startup, functional test)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment operates to manufacturer spec under static and functional test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commissioning Agent witness test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Month 12-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level 3-4 Commissioning (integrated systems, simulated load/failure)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power/cooling failover performs to design under simulated utility failure and full IT load</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final punch-list walkthrough</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Closeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No open life-safety items; all other items logged with an owner and due date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joint GC / IT Ops walkthrough</t>
+  </si>
+  <si>
     <t xml:space="preserve">RACI Matrix  (R = Responsible · A = Accountable · C = Consulted · I = Informed)</t>
   </si>
   <si>
@@ -492,9 +568,6 @@
   </si>
   <si>
     <t xml:space="preserve">Description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category</t>
   </si>
   <si>
     <t xml:space="preserve">Probability (1-5)</t>
@@ -2099,11 +2172,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2119,186 +2197,140 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>12</v>
+        <v>102</v>
       </c>
       <c r="B2" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="G7" s="10" t="s">
         <v>31</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2320,6 +2352,227 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>135</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2332,7 +2585,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -2342,82 +2595,82 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>118</v>
+        <v>143</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>119</v>
+        <v>144</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>133</v>
+        <v>158</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>134</v>
+        <v>159</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>135</v>
+        <v>160</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2425,79 +2678,79 @@
         <v>23</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>138</v>
+        <v>163</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>139</v>
+        <v>164</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>141</v>
+        <v>166</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>142</v>
+        <v>167</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>143</v>
+        <v>168</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>139</v>
+        <v>164</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>144</v>
+        <v>169</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>145</v>
+        <v>170</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>146</v>
+        <v>171</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>147</v>
+        <v>172</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>139</v>
+        <v>164</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>148</v>
+        <v>173</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>149</v>
+        <v>174</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>150</v>
+        <v>175</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>151</v>
+        <v>176</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -2514,7 +2767,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2535,7 +2788,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>152</v>
+        <v>177</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -2548,25 +2801,25 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>153</v>
+        <v>178</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>154</v>
+        <v>179</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>155</v>
+        <v>103</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>156</v>
+        <v>180</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>157</v>
+        <v>181</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>158</v>
+        <v>182</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>159</v>
+        <v>183</v>
       </c>
       <c r="H2" s="9" t="s">
         <v>13</v>
@@ -2577,13 +2830,13 @@
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>160</v>
+        <v>184</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>161</v>
+        <v>185</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>162</v>
+        <v>186</v>
       </c>
       <c r="D3" s="10" t="n">
         <v>2</v>
@@ -2596,24 +2849,24 @@
         <v>10</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>163</v>
+        <v>187</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>165</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>166</v>
+        <v>190</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>167</v>
+        <v>191</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>3</v>
@@ -2626,24 +2879,24 @@
         <v>12</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>169</v>
+        <v>193</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>31</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>170</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>171</v>
+        <v>195</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>172</v>
+        <v>196</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="D5" s="10" t="n">
         <v>4</v>
@@ -2656,24 +2909,24 @@
         <v>16</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>173</v>
+        <v>197</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>175</v>
+        <v>199</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>3</v>
@@ -2686,24 +2939,24 @@
         <v>9</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>36</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>165</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>180</v>
+        <v>204</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>181</v>
+        <v>205</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>2</v>
@@ -2716,24 +2969,24 @@
         <v>8</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>182</v>
+        <v>206</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>36</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>165</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>183</v>
+        <v>207</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>184</v>
+        <v>208</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="D8" s="11" t="n">
         <v>3</v>
@@ -2746,24 +2999,24 @@
         <v>9</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>186</v>
+        <v>210</v>
       </c>
       <c r="H8" s="11" t="s">
         <v>31</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>170</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>187</v>
+        <v>211</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>188</v>
+        <v>212</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>189</v>
+        <v>213</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>2</v>
@@ -2776,13 +3029,13 @@
         <v>6</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>190</v>
+        <v>214</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>191</v>
+        <v>215</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>170</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -2799,7 +3052,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2819,7 +3072,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>192</v>
+        <v>216</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -2831,39 +3084,39 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>193</v>
+        <v>217</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>194</v>
+        <v>218</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>154</v>
+        <v>179</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>195</v>
+        <v>219</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>196</v>
+        <v>220</v>
       </c>
       <c r="G2" s="9" t="s">
         <v>18</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>197</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>198</v>
+        <v>222</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>199</v>
+        <v>223</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>200</v>
+        <v>224</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>56</v>
@@ -2872,24 +3125,24 @@
         <v>31</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>201</v>
+        <v>225</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>203</v>
+        <v>227</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>199</v>
+        <v>223</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>204</v>
+        <v>228</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>46</v>
@@ -2898,39 +3151,39 @@
         <v>36</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>205</v>
+        <v>229</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>206</v>
+        <v>230</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>207</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>208</v>
+        <v>232</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>209</v>
+        <v>233</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>210</v>
+        <v>234</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>46</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>205</v>
+        <v>229</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>211</v>
+        <v>235</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>212</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -2947,7 +3200,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2965,7 +3218,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>213</v>
+        <v>237</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -2976,13 +3229,13 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>214</v>
+        <v>238</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>215</v>
+        <v>239</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>14</v>
@@ -2991,18 +3244,18 @@
         <v>15</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>217</v>
+        <v>241</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>218</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>219</v>
+        <v>243</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>220</v>
+        <v>244</v>
       </c>
       <c r="C3" s="12" t="n">
         <v>2450000</v>
@@ -3014,64 +3267,64 @@
         <v>79</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>221</v>
+        <v>245</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>222</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>223</v>
+        <v>247</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>224</v>
+        <v>248</v>
       </c>
       <c r="C4" s="14" t="n">
         <v>1450000</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>225</v>
+        <v>249</v>
       </c>
       <c r="E4" s="11" t="s">
         <v>67</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>221</v>
+        <v>245</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>222</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>226</v>
+        <v>250</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>227</v>
+        <v>251</v>
       </c>
       <c r="C5" s="12" t="n">
         <v>980000</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>225</v>
+        <v>249</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>67</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>221</v>
+        <v>245</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>222</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>228</v>
+        <v>252</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>229</v>
+        <v>253</v>
       </c>
       <c r="C6" s="14" t="n">
         <v>190000</v>
@@ -3083,18 +3336,18 @@
         <v>61</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>230</v>
+        <v>254</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>222</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>231</v>
+        <v>255</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>232</v>
+        <v>256</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>130000</v>
@@ -3106,18 +3359,18 @@
         <v>79</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>221</v>
+        <v>245</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>222</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>233</v>
+        <v>257</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>234</v>
+        <v>258</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>890000</v>
@@ -3129,10 +3382,10 @@
         <v>72</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>235</v>
+        <v>259</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>222</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>

</xml_diff>